<commit_message>
docs: add data/processed/README.md and update root README.md with spreadsheet format documentation
</commit_message>
<xml_diff>
--- a/data/evaluation_results.xlsx
+++ b/data/evaluation_results.xlsx
@@ -607,13 +607,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.820561501663178</v>
+        <v>1.655734999803826</v>
       </c>
       <c r="C12" t="n">
-        <v>1.857570499996655</v>
+        <v>1.530250995419919</v>
       </c>
       <c r="D12" t="n">
-        <v>1.871773495804518</v>
+        <v>1.469248002395034</v>
       </c>
     </row>
     <row r="13">
@@ -623,13 +623,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3863147998927161</v>
+        <v>0.3481285999296233</v>
       </c>
       <c r="C13" t="n">
-        <v>0.391080200090073</v>
+        <v>0.3215850000269711</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3959005000069737</v>
+        <v>0.3084874999476597</v>
       </c>
     </row>
   </sheetData>

</xml_diff>